<commit_message>
truss topology solving distributed load added
</commit_message>
<xml_diff>
--- a/OpeningAndSaving/Test.xlsx
+++ b/OpeningAndSaving/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5c2fbe8304562b3/Desktop/Structural_Analysis_Programing/Structural_Solver/OpeningAndSaving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{976152EE-7D44-47BA-920C-E335D656805B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD9A5FA5-2231-477C-BA77-BF5AA1FC8FF4}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{48DAB0DD-CC8D-4F5A-A391-266DF5B21CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45C07AFE-EA4E-4A1C-AEA9-055718A8CFAD}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="3135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Boundary" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>X</t>
   </si>
@@ -67,6 +67,54 @@
   </si>
   <si>
     <t>LoadCase2 fy</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis1x</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis1y</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis2x</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis2y</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis1fx</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis1fy</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis2fx</t>
+  </si>
+  <si>
+    <t>LoadCase1 dis2dy</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis1x</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis1y</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis1fx</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis1fy</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis2x</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis2y</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis2fx</t>
+  </si>
+  <si>
+    <t>LoadCase2 dis2dy</t>
   </si>
 </sst>
 </file>
@@ -119,10 +167,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -388,10 +432,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:AG68"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,36 +443,1524 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>222</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>282</v>
+      </c>
+      <c r="L2">
+        <v>12</v>
+      </c>
+      <c r="N2">
+        <v>72</v>
+      </c>
+      <c r="O2">
+        <v>5</v>
+      </c>
+      <c r="Q2">
+        <v>156</v>
+      </c>
+      <c r="R2">
+        <v>5</v>
+      </c>
+      <c r="T2">
+        <v>12</v>
+      </c>
+      <c r="U2">
+        <v>5</v>
+      </c>
+      <c r="W2">
+        <v>76</v>
+      </c>
+      <c r="X2">
+        <v>12</v>
+      </c>
+      <c r="Z2">
+        <v>160</v>
+      </c>
+      <c r="AA2">
+        <v>5</v>
+      </c>
+      <c r="AC2">
+        <v>238</v>
+      </c>
+      <c r="AD2">
+        <v>12</v>
+      </c>
+      <c r="AF2">
+        <v>4</v>
+      </c>
+      <c r="AG2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.4">
       <c r="A3">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>222</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>282</v>
+      </c>
+      <c r="L3">
+        <v>14</v>
+      </c>
+      <c r="N3">
+        <v>72</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="Q3">
+        <v>156</v>
+      </c>
+      <c r="R3">
+        <v>6</v>
+      </c>
+      <c r="T3">
+        <v>16</v>
+      </c>
+      <c r="U3">
+        <v>5</v>
+      </c>
+      <c r="W3">
+        <v>80</v>
+      </c>
+      <c r="X3">
+        <v>12</v>
+      </c>
+      <c r="Z3">
+        <v>164</v>
+      </c>
+      <c r="AA3">
+        <v>5</v>
+      </c>
+      <c r="AC3">
+        <v>242</v>
+      </c>
+      <c r="AD3">
+        <v>12</v>
+      </c>
+      <c r="AF3">
+        <v>8</v>
+      </c>
+      <c r="AG3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>222</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="K4">
+        <v>282</v>
+      </c>
+      <c r="L4">
+        <v>16</v>
+      </c>
+      <c r="N4">
+        <v>72</v>
+      </c>
+      <c r="O4">
+        <v>8</v>
+      </c>
+      <c r="Q4">
+        <v>156</v>
+      </c>
+      <c r="R4">
+        <v>8</v>
+      </c>
+      <c r="T4">
+        <v>20</v>
+      </c>
+      <c r="U4">
+        <v>5</v>
+      </c>
+      <c r="W4">
+        <v>84</v>
+      </c>
+      <c r="X4">
+        <v>12</v>
+      </c>
+      <c r="Z4">
+        <v>168</v>
+      </c>
+      <c r="AA4">
+        <v>5</v>
+      </c>
+      <c r="AC4">
+        <v>246</v>
+      </c>
+      <c r="AD4">
+        <v>12</v>
+      </c>
+      <c r="AF4">
+        <v>16</v>
+      </c>
+      <c r="AG4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>72</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>222</v>
+      </c>
+      <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>282</v>
+      </c>
+      <c r="L5">
+        <v>18</v>
+      </c>
+      <c r="N5">
+        <v>72</v>
+      </c>
+      <c r="O5">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A4">
+      <c r="Q5">
+        <v>156</v>
+      </c>
+      <c r="R5">
         <v>10</v>
       </c>
-      <c r="B4">
+      <c r="T5">
+        <v>24</v>
+      </c>
+      <c r="U5">
+        <v>5</v>
+      </c>
+      <c r="W5">
+        <v>88</v>
+      </c>
+      <c r="X5">
+        <v>12</v>
+      </c>
+      <c r="Z5">
+        <v>172</v>
+      </c>
+      <c r="AA5">
+        <v>5</v>
+      </c>
+      <c r="AC5">
+        <v>250</v>
+      </c>
+      <c r="AD5">
+        <v>12</v>
+      </c>
+      <c r="AF5">
+        <v>20</v>
+      </c>
+      <c r="AG5">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>72</v>
+      </c>
+      <c r="B6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="H6">
+        <v>222</v>
+      </c>
+      <c r="I6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>282</v>
+      </c>
+      <c r="L6">
+        <v>20</v>
+      </c>
+      <c r="N6">
+        <v>72</v>
+      </c>
+      <c r="O6">
+        <v>12</v>
+      </c>
+      <c r="Q6">
+        <v>156</v>
+      </c>
+      <c r="R6">
+        <v>12</v>
+      </c>
+      <c r="T6">
+        <v>28</v>
+      </c>
+      <c r="U6">
+        <v>5</v>
+      </c>
+      <c r="W6">
+        <v>92</v>
+      </c>
+      <c r="X6">
+        <v>12</v>
+      </c>
+      <c r="Z6">
+        <v>176</v>
+      </c>
+      <c r="AA6">
+        <v>5</v>
+      </c>
+      <c r="AC6">
+        <v>254</v>
+      </c>
+      <c r="AD6">
+        <v>12</v>
+      </c>
+      <c r="AF6">
+        <v>24</v>
+      </c>
+      <c r="AG6">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>156</v>
+      </c>
+      <c r="B7">
+        <v>12</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A5">
+      <c r="H7">
+        <v>222</v>
+      </c>
+      <c r="I7">
         <v>10</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="K7">
+        <v>282</v>
+      </c>
+      <c r="L7">
+        <v>22</v>
+      </c>
+      <c r="N7">
+        <v>72</v>
+      </c>
+      <c r="O7">
+        <v>14</v>
+      </c>
+      <c r="Q7">
+        <v>156</v>
+      </c>
+      <c r="R7">
+        <v>14</v>
+      </c>
+      <c r="T7">
+        <v>32</v>
+      </c>
+      <c r="U7">
+        <v>5</v>
+      </c>
+      <c r="W7">
+        <v>96</v>
+      </c>
+      <c r="X7">
+        <v>12</v>
+      </c>
+      <c r="Z7">
+        <v>180</v>
+      </c>
+      <c r="AA7">
+        <v>5</v>
+      </c>
+      <c r="AC7">
+        <v>258</v>
+      </c>
+      <c r="AD7">
+        <v>12</v>
+      </c>
+      <c r="AF7">
+        <v>28</v>
+      </c>
+      <c r="AG7">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>156</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="H8">
+        <v>222</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="K8">
+        <v>282</v>
+      </c>
+      <c r="L8">
+        <v>24</v>
+      </c>
+      <c r="N8">
+        <v>72</v>
+      </c>
+      <c r="O8">
+        <v>16</v>
+      </c>
+      <c r="Q8">
+        <v>156</v>
+      </c>
+      <c r="R8">
+        <v>16</v>
+      </c>
+      <c r="T8">
+        <v>36</v>
+      </c>
+      <c r="U8">
+        <v>5</v>
+      </c>
+      <c r="W8">
+        <v>100</v>
+      </c>
+      <c r="X8">
+        <v>12</v>
+      </c>
+      <c r="Z8">
+        <v>184</v>
+      </c>
+      <c r="AA8">
+        <v>5</v>
+      </c>
+      <c r="AC8">
+        <v>262</v>
+      </c>
+      <c r="AD8">
+        <v>12</v>
+      </c>
+      <c r="AF8">
+        <v>32</v>
+      </c>
+      <c r="AG8">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A9">
+        <v>222</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>14</v>
+      </c>
+      <c r="H9">
+        <v>222</v>
+      </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
+      <c r="K9">
+        <v>282</v>
+      </c>
+      <c r="L9">
+        <v>26</v>
+      </c>
+      <c r="N9">
+        <v>72</v>
+      </c>
+      <c r="O9">
+        <v>18</v>
+      </c>
+      <c r="Q9">
+        <v>156</v>
+      </c>
+      <c r="R9">
+        <v>18</v>
+      </c>
+      <c r="T9">
+        <v>40</v>
+      </c>
+      <c r="U9">
+        <v>5</v>
+      </c>
+      <c r="W9">
+        <v>104</v>
+      </c>
+      <c r="X9">
+        <v>12</v>
+      </c>
+      <c r="Z9">
+        <v>188</v>
+      </c>
+      <c r="AA9">
+        <v>5</v>
+      </c>
+      <c r="AC9">
+        <v>266</v>
+      </c>
+      <c r="AD9">
+        <v>12</v>
+      </c>
+      <c r="AF9">
+        <v>36</v>
+      </c>
+      <c r="AG9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A10">
+        <v>222</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>16</v>
+      </c>
+      <c r="H10">
+        <v>222</v>
+      </c>
+      <c r="I10">
+        <v>16</v>
+      </c>
+      <c r="N10">
+        <v>72</v>
+      </c>
+      <c r="O10">
+        <v>20</v>
+      </c>
+      <c r="Q10">
+        <v>156</v>
+      </c>
+      <c r="R10">
+        <v>20</v>
+      </c>
+      <c r="T10">
+        <v>44</v>
+      </c>
+      <c r="U10">
+        <v>5</v>
+      </c>
+      <c r="W10">
+        <v>108</v>
+      </c>
+      <c r="X10">
+        <v>12</v>
+      </c>
+      <c r="Z10">
+        <v>192</v>
+      </c>
+      <c r="AA10">
+        <v>5</v>
+      </c>
+      <c r="AC10">
+        <v>270</v>
+      </c>
+      <c r="AD10">
+        <v>12</v>
+      </c>
+      <c r="AF10">
+        <v>40</v>
+      </c>
+      <c r="AG10">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A11">
+        <v>234</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>18</v>
+      </c>
+      <c r="H11">
+        <v>222</v>
+      </c>
+      <c r="I11">
+        <v>18</v>
+      </c>
+      <c r="N11">
+        <v>72</v>
+      </c>
+      <c r="O11">
+        <v>22</v>
+      </c>
+      <c r="Q11">
+        <v>156</v>
+      </c>
+      <c r="R11">
+        <v>22</v>
+      </c>
+      <c r="T11">
+        <v>48</v>
+      </c>
+      <c r="U11">
+        <v>5</v>
+      </c>
+      <c r="W11">
+        <v>112</v>
+      </c>
+      <c r="X11">
+        <v>12</v>
+      </c>
+      <c r="Z11">
+        <v>196</v>
+      </c>
+      <c r="AA11">
+        <v>5</v>
+      </c>
+      <c r="AC11">
+        <v>274</v>
+      </c>
+      <c r="AD11">
+        <v>12</v>
+      </c>
+      <c r="AF11">
+        <v>44</v>
+      </c>
+      <c r="AG11">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A12">
+        <v>234</v>
+      </c>
+      <c r="B12">
+        <v>12</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>20</v>
+      </c>
+      <c r="H12">
+        <v>222</v>
+      </c>
+      <c r="I12">
+        <v>20</v>
+      </c>
+      <c r="N12">
+        <v>72</v>
+      </c>
+      <c r="O12">
+        <v>24</v>
+      </c>
+      <c r="Q12">
+        <v>156</v>
+      </c>
+      <c r="R12">
+        <v>24</v>
+      </c>
+      <c r="T12">
+        <v>52</v>
+      </c>
+      <c r="U12">
+        <v>5</v>
+      </c>
+      <c r="W12">
+        <v>116</v>
+      </c>
+      <c r="X12">
+        <v>12</v>
+      </c>
+      <c r="Z12">
+        <v>200</v>
+      </c>
+      <c r="AA12">
+        <v>5</v>
+      </c>
+      <c r="AC12">
+        <v>278</v>
+      </c>
+      <c r="AD12">
+        <v>12</v>
+      </c>
+      <c r="AF12">
+        <v>48</v>
+      </c>
+      <c r="AG12">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A13">
+        <v>282</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>22</v>
+      </c>
+      <c r="H13">
+        <v>222</v>
+      </c>
+      <c r="I13">
+        <v>22</v>
+      </c>
+      <c r="N13">
+        <v>72</v>
+      </c>
+      <c r="O13">
+        <v>26</v>
+      </c>
+      <c r="Q13">
+        <v>156</v>
+      </c>
+      <c r="R13">
+        <v>26</v>
+      </c>
+      <c r="T13">
+        <v>56</v>
+      </c>
+      <c r="U13">
+        <v>5</v>
+      </c>
+      <c r="W13">
+        <v>120</v>
+      </c>
+      <c r="X13">
+        <v>12</v>
+      </c>
+      <c r="Z13">
+        <v>204</v>
+      </c>
+      <c r="AA13">
+        <v>5</v>
+      </c>
+      <c r="AF13">
+        <v>52</v>
+      </c>
+      <c r="AG13">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A14">
+        <v>282</v>
+      </c>
+      <c r="B14">
+        <v>26</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>24</v>
+      </c>
+      <c r="H14">
+        <v>222</v>
+      </c>
+      <c r="I14">
+        <v>24</v>
+      </c>
+      <c r="T14">
+        <v>60</v>
+      </c>
+      <c r="U14">
+        <v>5</v>
+      </c>
+      <c r="W14">
+        <v>124</v>
+      </c>
+      <c r="X14">
+        <v>12</v>
+      </c>
+      <c r="Z14">
+        <v>208</v>
+      </c>
+      <c r="AA14">
+        <v>5</v>
+      </c>
+      <c r="AF14">
+        <v>56</v>
+      </c>
+      <c r="AG14">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15">
+        <v>26</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>26</v>
+      </c>
+      <c r="H15">
+        <v>222</v>
+      </c>
+      <c r="I15">
+        <v>26</v>
+      </c>
+      <c r="T15">
+        <v>64</v>
+      </c>
+      <c r="U15">
+        <v>5</v>
+      </c>
+      <c r="W15">
+        <v>128</v>
+      </c>
+      <c r="X15">
+        <v>12</v>
+      </c>
+      <c r="Z15">
+        <v>212</v>
+      </c>
+      <c r="AA15">
+        <v>5</v>
+      </c>
+      <c r="AF15">
+        <v>60</v>
+      </c>
+      <c r="AG15">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.4">
+      <c r="E16">
+        <v>12</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>234</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>68</v>
+      </c>
+      <c r="U16">
+        <v>5</v>
+      </c>
+      <c r="W16">
+        <v>132</v>
+      </c>
+      <c r="X16">
+        <v>12</v>
+      </c>
+      <c r="Z16">
+        <v>216</v>
+      </c>
+      <c r="AA16">
+        <v>5</v>
+      </c>
+      <c r="AF16">
+        <v>64</v>
+      </c>
+      <c r="AG16">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E17">
+        <v>12</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="H17">
+        <v>234</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+      <c r="W17">
+        <v>136</v>
+      </c>
+      <c r="X17">
+        <v>12</v>
+      </c>
+      <c r="Z17">
+        <v>220</v>
+      </c>
+      <c r="AA17">
+        <v>5</v>
+      </c>
+      <c r="AF17">
+        <v>68</v>
+      </c>
+      <c r="AG17">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E18">
+        <v>12</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="H18">
+        <v>234</v>
+      </c>
+      <c r="I18">
+        <v>4</v>
+      </c>
+      <c r="W18">
+        <v>140</v>
+      </c>
+      <c r="X18">
+        <v>12</v>
+      </c>
+      <c r="AF18">
+        <v>76</v>
+      </c>
+      <c r="AG18">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E19">
+        <v>12</v>
+      </c>
+      <c r="F19">
+        <v>6</v>
+      </c>
+      <c r="H19">
+        <v>234</v>
+      </c>
+      <c r="I19">
+        <v>6</v>
+      </c>
+      <c r="W19">
+        <v>144</v>
+      </c>
+      <c r="X19">
+        <v>12</v>
+      </c>
+      <c r="AF19">
+        <v>80</v>
+      </c>
+      <c r="AG19">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E20">
+        <v>12</v>
+      </c>
+      <c r="F20">
+        <v>8</v>
+      </c>
+      <c r="H20">
+        <v>234</v>
+      </c>
+      <c r="I20">
+        <v>8</v>
+      </c>
+      <c r="W20">
+        <v>148</v>
+      </c>
+      <c r="X20">
+        <v>12</v>
+      </c>
+      <c r="AF20">
+        <v>84</v>
+      </c>
+      <c r="AG20">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E21">
+        <v>12</v>
+      </c>
+      <c r="F21">
+        <v>10</v>
+      </c>
+      <c r="H21">
+        <v>234</v>
+      </c>
+      <c r="I21">
+        <v>10</v>
+      </c>
+      <c r="W21">
+        <v>152</v>
+      </c>
+      <c r="X21">
+        <v>12</v>
+      </c>
+      <c r="AF21">
+        <v>88</v>
+      </c>
+      <c r="AG21">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E22">
+        <v>12</v>
+      </c>
+      <c r="F22">
+        <v>12</v>
+      </c>
+      <c r="H22">
+        <v>234</v>
+      </c>
+      <c r="I22">
+        <v>12</v>
+      </c>
+      <c r="AF22">
+        <v>92</v>
+      </c>
+      <c r="AG22">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E23">
+        <v>12</v>
+      </c>
+      <c r="F23">
+        <v>14</v>
+      </c>
+      <c r="H23">
+        <v>234</v>
+      </c>
+      <c r="I23">
+        <v>14</v>
+      </c>
+      <c r="AF23">
+        <v>96</v>
+      </c>
+      <c r="AG23">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E24">
+        <v>12</v>
+      </c>
+      <c r="F24">
+        <v>16</v>
+      </c>
+      <c r="H24">
+        <v>234</v>
+      </c>
+      <c r="I24">
+        <v>16</v>
+      </c>
+      <c r="AF24">
+        <v>100</v>
+      </c>
+      <c r="AG24">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E25">
+        <v>12</v>
+      </c>
+      <c r="F25">
+        <v>18</v>
+      </c>
+      <c r="H25">
+        <v>234</v>
+      </c>
+      <c r="I25">
+        <v>18</v>
+      </c>
+      <c r="AF25">
+        <v>104</v>
+      </c>
+      <c r="AG25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E26">
+        <v>12</v>
+      </c>
+      <c r="F26">
+        <v>20</v>
+      </c>
+      <c r="H26">
+        <v>234</v>
+      </c>
+      <c r="I26">
+        <v>20</v>
+      </c>
+      <c r="AF26">
+        <v>108</v>
+      </c>
+      <c r="AG26">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E27">
+        <v>12</v>
+      </c>
+      <c r="F27">
+        <v>22</v>
+      </c>
+      <c r="H27">
+        <v>234</v>
+      </c>
+      <c r="I27">
+        <v>22</v>
+      </c>
+      <c r="AF27">
+        <v>112</v>
+      </c>
+      <c r="AG27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E28">
+        <v>12</v>
+      </c>
+      <c r="F28">
+        <v>24</v>
+      </c>
+      <c r="H28">
+        <v>234</v>
+      </c>
+      <c r="I28">
+        <v>24</v>
+      </c>
+      <c r="AF28">
+        <v>116</v>
+      </c>
+      <c r="AG28">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="E29">
+        <v>12</v>
+      </c>
+      <c r="F29">
+        <v>26</v>
+      </c>
+      <c r="H29">
+        <v>234</v>
+      </c>
+      <c r="I29">
+        <v>26</v>
+      </c>
+      <c r="AF29">
+        <v>120</v>
+      </c>
+      <c r="AG29">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="AF30">
+        <v>124</v>
+      </c>
+      <c r="AG30">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="AF31">
+        <v>128</v>
+      </c>
+      <c r="AG31">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="5:33" x14ac:dyDescent="0.4">
+      <c r="AF32">
+        <v>132</v>
+      </c>
+      <c r="AG32">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF33">
+        <v>136</v>
+      </c>
+      <c r="AG33">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF34">
+        <v>140</v>
+      </c>
+      <c r="AG34">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF35">
+        <v>144</v>
+      </c>
+      <c r="AG35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF36">
+        <v>148</v>
+      </c>
+      <c r="AG36">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF37">
+        <v>152</v>
+      </c>
+      <c r="AG37">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF38">
+        <v>160</v>
+      </c>
+      <c r="AG38">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF39">
+        <v>164</v>
+      </c>
+      <c r="AG39">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF40">
+        <v>168</v>
+      </c>
+      <c r="AG40">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF41">
+        <v>172</v>
+      </c>
+      <c r="AG41">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF42">
+        <v>176</v>
+      </c>
+      <c r="AG42">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF43">
+        <v>180</v>
+      </c>
+      <c r="AG43">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF44">
+        <v>184</v>
+      </c>
+      <c r="AG44">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF45">
+        <v>188</v>
+      </c>
+      <c r="AG45">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF46">
+        <v>192</v>
+      </c>
+      <c r="AG46">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF47">
+        <v>196</v>
+      </c>
+      <c r="AG47">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF48">
+        <v>200</v>
+      </c>
+      <c r="AG48">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF49">
+        <v>204</v>
+      </c>
+      <c r="AG49">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF50">
+        <v>208</v>
+      </c>
+      <c r="AG50">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF51">
+        <v>212</v>
+      </c>
+      <c r="AG51">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF52">
+        <v>216</v>
+      </c>
+      <c r="AG52">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF53">
+        <v>220</v>
+      </c>
+      <c r="AG53">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF54">
+        <v>224</v>
+      </c>
+      <c r="AG54">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF55">
+        <v>228</v>
+      </c>
+      <c r="AG55">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF56">
+        <v>232</v>
+      </c>
+      <c r="AG56">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF57">
+        <v>236</v>
+      </c>
+      <c r="AG57">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF58">
+        <v>240</v>
+      </c>
+      <c r="AG58">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF59">
+        <v>244</v>
+      </c>
+      <c r="AG59">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF60">
+        <v>248</v>
+      </c>
+      <c r="AG60">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF61">
+        <v>252</v>
+      </c>
+      <c r="AG61">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF62">
+        <v>256</v>
+      </c>
+      <c r="AG62">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="63" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF63">
+        <v>260</v>
+      </c>
+      <c r="AG63">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF64">
+        <v>264</v>
+      </c>
+      <c r="AG64">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="65" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF65">
+        <v>268</v>
+      </c>
+      <c r="AG65">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="66" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF66">
+        <v>272</v>
+      </c>
+      <c r="AG66">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF67">
+        <v>276</v>
+      </c>
+      <c r="AG67">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="32:33" x14ac:dyDescent="0.4">
+      <c r="AF68">
+        <v>280</v>
+      </c>
+      <c r="AG68">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C87C47EB-3377-4B84-8A33-CCB727C23BA2}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="28.765625" customWidth="1"/>
@@ -536,9 +2068,11 @@
     <col min="3" max="3" width="13.53515625" customWidth="1"/>
     <col min="4" max="4" width="14.23046875" customWidth="1"/>
     <col min="5" max="5" width="16.61328125" customWidth="1"/>
+    <col min="6" max="6" width="16.3828125" customWidth="1"/>
+    <col min="7" max="7" width="14.765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -555,19 +2089,67 @@
         <v>5</v>
       </c>
       <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="O1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="P1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="Q1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>2</v>
       </c>
@@ -583,16 +2165,16 @@
       <c r="E2">
         <v>-5</v>
       </c>
-      <c r="F2">
+      <c r="N2">
         <v>10</v>
       </c>
-      <c r="G2">
-        <v>5</v>
-      </c>
-      <c r="H2">
+      <c r="O2">
+        <v>5</v>
+      </c>
+      <c r="P2">
         <v>-5</v>
       </c>
-      <c r="I2">
+      <c r="Q2">
         <v>0</v>
       </c>
     </row>

</xml_diff>